<commit_message>
Schematron updates for v3.5.1.251001CP2.
</commit_message>
<xml_diff>
--- a/Schematron/documentation/Schematron_3.5.0_3.5.1_Comparison.xlsx
+++ b/Schematron/documentation/Schematron_3.5.0_3.5.1_Comparison.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josh\Documents\NEMSIS TAC\Repository\nemsis_public\Schematron\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josh\Documents\NEMSIS TAC\Repository\nemsis\Schematron\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D78278D-F68C-4D05-95B2-5988F0EDC97E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B76A28-70F8-4A4C-8A50-7A91B052B5B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{EFB0DDD4-CF85-4C10-9AFB-9B88D9ECAAEF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="405">
   <si>
     <t>…</t>
   </si>
@@ -1247,13 +1247,10 @@
     <t>Sex should be recorded when Patient Evaluation/Care is "Patient Evaluated and Care Provided".</t>
   </si>
   <si>
-    <t>3.5.0.250403CP5</t>
-  </si>
-  <si>
-    <t>3.5.1.250403CP1</t>
-  </si>
-  <si>
-    <t>National Schematron Rules Comparison for EMSDataSet</t>
+    <t>3.5.0.251001CP6</t>
+  </si>
+  <si>
+    <t>3.5.1.251001CP2</t>
   </si>
 </sst>
 </file>
@@ -1879,7 +1876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91DB0597-B734-4DDE-A8D8-647079D1FCD6}">
-  <dimension ref="A1:G201"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.77734375" style="1" customWidth="1"/>
@@ -1894,7 +1891,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>405</v>
+        <v>384</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -3258,2551 +3255,2551 @@
         <v>252</v>
       </c>
     </row>
+    <row r="70" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A70" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
     <row r="71" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F73" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="E74" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F74" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G74" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F76" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F77" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F78" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F79" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F80" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F81" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F82" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F83" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F84" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F85" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="E86" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="F86" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G86" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+        <v>271</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G88" s="2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F89" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F90" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F91" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F92" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F93" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F94" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B95" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F95" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F96" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B97" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F97" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F98" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>281</v>
+        <v>376</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F99" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>281</v>
+        <v>376</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B100" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F100" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>377</v>
+        <v>282</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F101" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B102" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F102" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F103" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B104" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F104" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B105" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B106" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G106" s="2" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="107" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B107" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="108" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B108" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G108" s="2" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B109" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F109" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G109" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="110" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B110" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F110" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B111" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F111" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="112" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B112" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F112" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>387</v>
+        <v>293</v>
       </c>
     </row>
     <row r="113" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B113" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="114" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B114" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F114" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B115" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B116" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F116" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B117" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F117" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G117" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B118" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F118" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B119" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F119" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="120" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B120" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F120" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="121" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B121" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F121" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G121" s="2" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="122" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B122" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G122" s="2" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="123" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B123" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E123" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F123" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G123" s="2" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="124" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B124" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E124" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F124" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G124" s="2" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="125" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B125" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E125" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F125" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G125" s="2" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B126" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E126" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F126" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G126" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B127" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E127" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F127" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G127" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="128" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B128" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F128" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="129" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B129" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E129" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F129" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G129" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="130" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B130" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E130" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F130" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="131" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B131" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E131" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F131" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="132" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B132" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E132" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F132" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G132" s="2" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="133" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B133" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E133" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F133" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G133" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="134" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B134" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E134" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F134" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G134" s="2" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="135" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B135" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E135" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F135" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G135" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="136" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B136" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E136" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F136" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G136" s="2" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="137" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E137" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F137" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G137" s="2" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B138" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E138" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F138" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G138" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="139" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B139" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E139" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F139" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G139" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="140" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B140" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E140" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F140" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G140" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="141" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B141" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E141" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F141" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G141" s="2" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="142" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B142" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E142" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F142" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G142" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="143" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B143" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E143" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F143" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G143" s="2" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B144" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E144" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F144" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G144" s="2" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B145" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E145" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F145" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G145" s="2" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="146" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B146" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E146" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F146" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G146" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="147" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B147" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E147" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F147" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G147" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="148" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B148" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E148" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F148" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G148" s="2" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B149" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E149" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F149" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G149" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="150" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E150" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F150" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G150" s="2" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B151" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E151" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F151" s="1" t="s">
         <v>2</v>
       </c>
       <c r="G151" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="152" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B152" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E152" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F152" s="1" t="s">
         <v>2</v>
       </c>
       <c r="G152" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="153" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E153" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F153" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G153" s="2" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="154" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B154" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E154" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F154" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G154" s="2" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="155" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B155" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E155" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F155" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G155" s="2" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="156" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B156" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E156" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F156" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G156" s="2" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="157" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B157" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E157" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F157" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G157" s="2" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="158" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B158" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E158" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F158" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G158" s="2" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="159" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B159" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E159" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F159" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G159" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="160" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B160" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E160" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F160" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G160" s="2" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="161" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B161" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E161" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F161" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G161" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="162" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B162" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E162" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F162" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G162" s="2" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="163" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B163" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E163" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F163" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G163" s="2" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="164" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B164" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E164" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F164" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G164" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="165" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B165" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E165" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F165" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G165" s="2" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="166" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B166" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E166" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F166" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G166" s="2" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="167" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B167" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E167" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F167" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G167" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="168" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A168" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B168" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E168" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F168" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G168" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="169" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A169" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B169" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E169" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F169" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G169" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="170" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B170" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E170" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F170" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G170" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="171" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B171" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E171" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F171" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G171" s="2" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="172" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B172" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E172" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F172" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G172" s="2" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="173" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B173" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E173" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F173" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G173" s="2" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="174" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A174" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B174" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E174" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F174" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G174" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="175" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A175" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B175" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E175" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F175" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G175" s="2" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="176" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A176" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B176" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E176" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F176" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G176" s="2" t="s">
-        <v>388</v>
+        <v>357</v>
       </c>
     </row>
     <row r="177" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B177" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E177" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F177" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G177" s="2" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="178" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A178" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B178" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E178" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F178" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G178" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="179" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A179" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B179" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E179" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F179" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G179" s="2" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="180" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A180" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B180" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E180" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F180" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G180" s="2" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="181" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A181" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B181" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E181" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F181" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G181" s="2" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="182" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A182" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B182" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E182" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F182" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G182" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="183" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A183" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B183" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E183" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F183" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G183" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="184" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A184" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B184" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E184" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F184" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G184" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="185" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A185" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B185" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E185" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F185" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G185" s="2" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="186" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A186" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B186" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E186" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F186" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G186" s="2" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="187" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A187" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B187" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E187" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F187" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G187" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="188" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A188" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B188" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E188" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F188" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G188" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="189" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A189" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B189" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E189" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F189" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G189" s="2" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="190" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A190" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B190" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E190" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F190" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G190" s="2" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="191" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A191" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B191" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E191" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F191" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G191" s="2" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="192" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A192" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B192" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E192" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F192" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G192" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="193" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A193" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B193" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E193" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F193" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G193" s="2" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="194" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A194" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B194" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E194" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F194" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G194" s="2" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="195" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A195" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="B195" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C195" s="2" t="s">
         <v>375</v>
       </c>
+    </row>
+    <row r="195" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="E195" s="1" t="s">
-        <v>189</v>
+        <v>389</v>
       </c>
       <c r="F195" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G195" s="2" t="s">
-        <v>375</v>
+        <v>394</v>
       </c>
     </row>
     <row r="196" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="E196" s="1" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F196" s="1" t="s">
         <v>2</v>
       </c>
       <c r="G196" s="2" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="197" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="E197" s="1" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F197" s="1" t="s">
         <v>2</v>
       </c>
       <c r="G197" s="2" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="198" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="E198" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F198" s="1" t="s">
         <v>2</v>
       </c>
       <c r="G198" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="199" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="E199" s="1" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F199" s="1" t="s">
         <v>2</v>
       </c>
       <c r="G199" s="2" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="200" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A200" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="B200" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C200" s="2" t="s">
+        <v>402</v>
+      </c>
       <c r="E200" s="1" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="F200" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G200" s="2" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="201" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A201" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="B201" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C201" s="2" t="s">
-        <v>402</v>
-      </c>
-      <c r="E201" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="F201" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G201" s="2" t="s">
         <v>402</v>
       </c>
     </row>
@@ -5812,13 +5809,13 @@
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="E2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A4:C69 A71:C201">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="notEqual">
+  <conditionalFormatting sqref="A4:C200">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="notEqual">
       <formula>E4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E4:G69 E71:G201">
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="notEqual">
+  <conditionalFormatting sqref="E4:G200">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="notEqual">
       <formula>A4</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>